<commit_message>
docs(entrepreneuriat): baseline of 15/10 and audit of @syntheza.eip
Instagram @syntheza.eip is the only network (5 followers, 6 posts, pre-pivot messaging, one unsourced figure); no LinkedIn page exists yet. Records the baseline in the KPI workbook, proposes a B2B bio and archiving four pre-pivot posts, and re-renders the CTA visuals with the real handle.
</commit_message>
<xml_diff>
--- a/entrepreneuriat/calendrier-editorial.xlsx
+++ b/entrepreneuriat/calendrier-editorial.xlsx
@@ -834,7 +834,7 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Compte Instagram Syntheza</t>
+          <t>Instagram @syntheza.eip</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1012,7 +1012,7 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Compte Instagram Syntheza</t>
+          <t>Instagram @syntheza.eip</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1190,7 +1190,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Compte Instagram Syntheza</t>
+          <t>Instagram @syntheza.eip</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>Compte Instagram Syntheza</t>
+          <t>Instagram @syntheza.eip</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
@@ -1692,7 +1692,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Compte Instagram Syntheza</t>
+          <t>Instagram @syntheza.eip</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>Compte Instagram Syntheza</t>
+          <t>Instagram @syntheza.eip</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -2016,7 +2016,7 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Compte Instagram Syntheza</t>
+          <t>Instagram @syntheza.eip</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -2340,7 +2340,7 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>Compte Instagram Syntheza</t>
+          <t>Instagram @syntheza.eip</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -2591,7 +2591,7 @@
       </c>
       <c r="F25" s="8" t="inlineStr">
         <is>
-          <t>Compte Instagram Syntheza</t>
+          <t>Instagram @syntheza.eip</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr">
@@ -2838,7 +2838,7 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>Compte Instagram Syntheza</t>
+          <t>Instagram @syntheza.eip</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -3089,7 +3089,7 @@
       </c>
       <c r="F31" s="8" t="inlineStr">
         <is>
-          <t>Compte Instagram Syntheza</t>
+          <t>Instagram @syntheza.eip</t>
         </is>
       </c>
       <c r="G31" s="6" t="inlineStr">
@@ -3344,7 +3344,7 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>Compte Instagram Syntheza</t>
+          <t>Instagram @syntheza.eip</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -3680,7 +3680,7 @@
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>Compte Instagram Syntheza</t>
+          <t>Instagram @syntheza.eip</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -3931,7 +3931,7 @@
       </c>
       <c r="F41" s="8" t="inlineStr">
         <is>
-          <t>Compte Instagram Syntheza</t>
+          <t>Instagram @syntheza.eip</t>
         </is>
       </c>
       <c r="G41" s="6" t="inlineStr">
@@ -4267,7 +4267,7 @@
       </c>
       <c r="F45" s="8" t="inlineStr">
         <is>
-          <t>Compte Instagram Syntheza</t>
+          <t>Instagram @syntheza.eip</t>
         </is>
       </c>
       <c r="G45" s="6" t="inlineStr">
@@ -4518,7 +4518,7 @@
       </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>Compte Instagram Syntheza</t>
+          <t>Instagram @syntheza.eip</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -4769,7 +4769,7 @@
       </c>
       <c r="F51" s="8" t="inlineStr">
         <is>
-          <t>Compte Instagram Syntheza</t>
+          <t>Instagram @syntheza.eip</t>
         </is>
       </c>
       <c r="G51" s="6" t="inlineStr">
@@ -5097,7 +5097,7 @@
       </c>
       <c r="F55" s="8" t="inlineStr">
         <is>
-          <t>Compte Instagram Syntheza</t>
+          <t>Instagram @syntheza.eip</t>
         </is>
       </c>
       <c r="G55" s="6" t="inlineStr">
@@ -5425,7 +5425,7 @@
       </c>
       <c r="F59" s="8" t="inlineStr">
         <is>
-          <t>Compte Instagram Syntheza</t>
+          <t>Instagram @syntheza.eip</t>
         </is>
       </c>
       <c r="G59" s="6" t="inlineStr">
@@ -5676,7 +5676,7 @@
       </c>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t>Compte Instagram Syntheza</t>
+          <t>Instagram @syntheza.eip</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">

</xml_diff>